<commit_message>
Add persistent pulse tracking for VOLUME meters
Refactors the VOLUME TRAM2_G1 and TRAM4 firmware to persist pulse state in EEPROM, validate RTC time, queue daily totals for upload, and improve the Blynk API and pulse-filter logic. This also updates the relevant Blynk auth/configuration values for the devices, fixes the Kenh12 server URL/tokens, and refreshes the associated mailbox/account mappings.
</commit_message>
<xml_diff>
--- a/Cảm biến + Sim.xlsx
+++ b/Cảm biến + Sim.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/43e69fe3b798304f/Work/PIO/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="20" documentId="11_F25DC773A252ABDACC104887E15F42345ADE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C7A00BAB-7FDB-4A7E-973E-B13E6CFBF0B0}"/>
+  <xr:revisionPtr revIDLastSave="21" documentId="11_F25DC773A252ABDACC104887E15F42345ADE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6725E891-BFAE-4234-9FBD-23A11DF777FE}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4440" yWindow="5868" windowWidth="22332" windowHeight="10632" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="42">
   <si>
     <t>Zero</t>
   </si>
@@ -158,6 +158,9 @@
   </si>
   <si>
     <t>01698049699</t>
+  </si>
+  <si>
+    <t>BK1</t>
   </si>
 </sst>
 </file>
@@ -249,8 +252,8 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Bình thường" xfId="0" builtinId="0"/>
+    <cellStyle name="Siêu kết nối" xfId="1" builtinId="8"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -263,6 +266,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -661,6 +668,9 @@
       <c r="E6" s="3">
         <v>45865</v>
       </c>
+      <c r="F6" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B7" t="s">

</xml_diff>